<commit_message>
data: add 3 sources via SOP pilot pipeline (ids 42-44)
- EPA Enterprise Data Catalog (id 42) - tracking-sheet candidate was
  'EPA Environmental Dataset Gateway (EDG)'; EDG is retired and
  redirects to the Enterprise Data Catalog, entry renamed accordingly
- EPA AirData (id 43)
- Water Quality Portal (id 44)

New visible tags approved by Jonathan: Air Quality, Water Quality
(vocabulary now 19). Each entry: researched from the source's own
pages by a research agent, adversarially verified by a separate agent
(all links live, facts cited; fixes applied for a contradicted refresh
cadence, stale dataset count, and citation format), 123-129 invisible
tags, 5-section markdown popup. dateAdded stored as text date so the
Recently Added badge renders. Headless smoke test: 44 cards, 3 badges,
new tag filters work, zero page errors.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ufe9nc2JgwE6aqTK8tTzoB
</commit_message>
<xml_diff>
--- a/datasets.xlsx
+++ b/datasets.xlsx
@@ -4318,20 +4318,86 @@
       <c r="AB42" s="2" t="n"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
-      <c r="A43" s="1" t="n"/>
-      <c r="B43" s="1" t="n"/>
-      <c r="C43" s="1" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="1" t="n"/>
-      <c r="F43" s="1" t="n"/>
-      <c r="G43" s="1" t="n"/>
+      <c r="A43" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>EPA Enterprise Data Catalog</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>EPA's Enterprise Data Catalog indexes thousands of agency air, water, land, and chemical datasets for open discovery.</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.epa.gov/data/enterprise-data-catalog</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>People; Ecosystems</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
       <c r="H43" s="1" t="n"/>
-      <c r="I43" s="1" t="n"/>
-      <c r="J43" s="1" t="n"/>
-      <c r="K43" s="3" t="n"/>
-      <c r="L43" s="1" t="n"/>
-      <c r="M43" s="3" t="n"/>
-      <c r="N43" s="1" t="n"/>
+      <c r="I43" s="1" t="n">
+        <v>1901</v>
+      </c>
+      <c r="J43" s="1" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Ecosystem Data; Public Health; Air Quality; Water Quality; Land Management; Energy</t>
+        </is>
+      </c>
+      <c r="L43" s="1" t="inlineStr">
+        <is>
+          <t>EPA; U.S. EPA; US EPA; USEPA; United States Environmental Protection Agency; Environmental Protection Agency; Enterprise Data Catalog; EDC; Environmental Dataset Gateway; EDG; Data.gov; General Services Administration; GSA; Office of Mission Support; Office of Information Collection; open data; open government; metadata catalog; data inventory; federal data; government data; air quality; water quality; drinking water; watersheds; impaired waters; surface water; groundwater; greenhouse gas emissions; GHG inventory; emission factors; criteria pollutants; toxic chemical releases; Toxics Release Inventory; TRI; PCBs; pesticides; chemicals; chemical safety; hazardous waste; solid waste; Superfund; brownfields; contaminated sites; environmental justice; climate change; climate change indicators; ecosystem services; land cover; land use; facility compliance; enforcement data; ecotoxicology; ECOTOX; Envirofacts; EnviroAtlas; ECHO; Enforcement and Compliance History Online; AirNow; AirData; Air Quality System; AQS; ATTAINS; WATERS; Clean Air Markets; Facility Registry Service; FRS; System of Registries; Central Data Exchange; CDX; How's My Waterway; Clip and Ship; EPA GeoPlatform; GIS; geospatial data; geospatial analysis; shapefile; CSV; JSON; GeoJSON; XML; XLSX; ZIP; KML; REST API; web services; API; api.data.gov; API key; DCAT; FGDC; ISO 19115; metadata; CKAN; ArcGIS; ArcGIS Hub; Esri; environmental monitoring; exposure assessment; risk assessment; ecological risk assessment; environmental epidemiology; environmental toxicology; environmental compliance; environmental health; One Health; pollution; emissions; regulatory data; United States; nationwide; state-level; county-level; facility-level; EPA Regions; watershed data; Ecosystem Data; Public Health; Air Quality; Water Quality; Land Management; Energy; Historic; Current; Present; 1901-2026; continuously updated</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>The Enterprise Data Catalog is the U.S. Environmental Protection Agency's master inventory of open data; the former Environmental Dataset Gateway (EDG) now redirects here. Metadata records contributed by EPA program offices, regional offices, and research laboratories cover air, water, land, waste, chemicals, climate, and environmental-health topics, with the searchable catalog hosted on Data.gov (about 6,600 EPA datasets as of September 2026). Researchers can download data in common formats, extract custom geospatial subsets, browse bulk files by office and region, or query the agency's public APIs and web services.
+#### Host Organization
+- United States Environmental Protection Agency (U.S. EPA)
+#### Data Format
+- Formats vary by dataset; commonly:
+	- **Tabular/structured**: CSV, JSON, XLSX, XML, ZIP archives
+	- **Geospatial**: GeoJSON, KML, plus on-demand extraction via the Clip and Ship ArcGIS Hub
+- Nine public APIs and web services (e.g., AirData AQS, ECHO, WATERS, Facility Registry Service); some require a free api.data.gov key
+#### How to access data of interest
+- Orient at the [EPA Enterprise Data Catalog](https://www.epa.gov/data/enterprise-data-catalog), which links every access route
+- Search and filter EPA's inventory on [Data.gov](https://catalog.data.gov/organization/epa-gov) by keyword, tag, and format, then download from the dataset record - no login needed
+- Browse bulk files by EPA office and region at the [EPA Data Download Site](https://edg.epa.gov/data/public/) or pick an API from [EPA Data APIs](https://www.epa.gov/data/application-programming-interface-api)
+#### Database Time Range
+- 1901-2026
+	- Coverage varies by dataset; some historical series reach back to the early 1900s
+#### Access Type
+- Public
+#### Citation Information
+- EPA data is public domain by default under the [EPA Data License](https://edg.epa.gov/EPA_Data_License.html); cite individual datasets per their own metadata
+- U.S. Environmental Protection Agency. "Enterprise Data Catalog." *US EPA*, May 2026, &lt;https://www.epa.gov/data/enterprise-data-catalog&gt;. 2026-09-01
+- See specific source citation details on the database website.</t>
+        </is>
+      </c>
+      <c r="N43" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="O43" s="1" t="n"/>
       <c r="P43" s="1" t="n"/>
       <c r="Q43" s="1" t="n"/>
@@ -4348,20 +4414,85 @@
       <c r="AB43" s="2" t="n"/>
     </row>
     <row r="44" ht="14.25" customHeight="1">
-      <c r="A44" s="1" t="n"/>
-      <c r="B44" s="1" t="n"/>
-      <c r="C44" s="1" t="n"/>
-      <c r="D44" s="3" t="n"/>
-      <c r="E44" s="1" t="n"/>
-      <c r="F44" s="1" t="n"/>
-      <c r="G44" s="1" t="n"/>
+      <c r="A44" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>EPA AirData</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>AirData provides outdoor air quality data from thousands of monitors across the U.S. since 1980.</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.epa.gov/outdoor-air-quality-data</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>People; Ecosystems</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
       <c r="H44" s="1" t="n"/>
-      <c r="I44" s="1" t="n"/>
-      <c r="J44" s="1" t="n"/>
-      <c r="K44" s="3" t="n"/>
-      <c r="L44" s="1" t="n"/>
-      <c r="M44" s="3" t="n"/>
-      <c r="N44" s="1" t="n"/>
+      <c r="I44" s="1" t="n">
+        <v>1980</v>
+      </c>
+      <c r="J44" s="1" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Air Quality; Public Health; Population Health; Ecosystem Data; Weather</t>
+        </is>
+      </c>
+      <c r="L44" s="1" t="inlineStr">
+        <is>
+          <t>AirData; EPA AirData; Outdoor Air Quality Data; EPA; U.S. EPA; US EPA; USEPA; United States Environmental Protection Agency; Environmental Protection Agency; Office of Air and Radiation; OAR; OAQPS; state local and tribal air agencies; Air Quality System; AQS; AQS Data Mart; AQS API; AirNow; Fire and Smoke Map; Pre-generated Data Files; Download Daily Data; Daily Air Quality Tracker; Tile Plot; AQI Plot; Concentration Plot; Concentration Map; Air Quality Index Report; Monitor Values Report; air quality; air pollution; outdoor air; ambient air; air monitoring; PM2.5; PM10; particulate matter; fine particles; coarse particles; ozone; O3; ground-level ozone; carbon monoxide; CO; nitrogen dioxide; NO2; sulfur dioxide; SO2; lead; Pb; criteria pollutants; criteria gases; hazardous air pollutants; HAPs; air toxics; VOCs; volatile organic compounds; ozone precursors; PM speciation; AQI; Air Quality Index; NAAQS; National Ambient Air Quality Standards; design values; total suspended particulate; TSP; meteorological data; wind; temperature; humidity; barometric pressure; smoke; wildfire smoke; emissions; smog; haze; visibility; CSV; ZIP; JSON; REST API; API key; OpenAPI; interactive maps; charts; reports; air quality monitoring; air pollution epidemiology; exposure assessment; environmental epidemiology; atmospheric science; environmental monitoring; respiratory health; asthma; cardiovascular health; environmental justice; trend analysis; regulatory data; United States; USA; nationwide; Puerto Rico; U.S. Virgin Islands; state; county; city; CBSA; monitoring site; outdoor monitors; Air Quality; Public Health; Population Health; Ecosystem Data; Weather; Historic; Current; Present; 1980-2026; 1957; hourly data; daily summaries; annual summaries; ozone season; updated semiannually</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>AirData is EPA's public gateway to the Air Quality System (AQS), the agency's repository of ambient air measurements reported by EPA, state, local, and tribal agencies at thousands of outdoor monitors across the United States, Puerto Rico, and the U.S. Virgin Islands. It offers pre-generated annual, daily, and hourly files for criteria pollutants, air toxics, and meteorological parameters from 1980 to the present, plus interactive query tools, AQI reports, visualizations, and an API for row-level data. These are the quality-assured measurements behind federal air standards; for real-time conditions, EPA points users to AirNow.
+#### Host Organization
+- United States Environmental Protection Agency (U.S. EPA)
+#### Data Format
+- **Pre-generated bulk files**: CSV in ZIP archives by pollutant and year (annual, daily, hourly)
+- **AQS API**: JSON REST web service for row-level sample data (free email registration for a key)
+- **Interactive tools**: filtered CSV extracts, AQI reports, and visualizations on the AirData site
+#### How to access data of interest
+- Start at [EPA AirData](https://www.epa.gov/outdoor-air-quality-data) and choose downloads, visualizations, or reports
+- For bulk data, open [Pre-generated Data Files](https://aqs.epa.gov/aqsweb/airdata/download_files.html), pick pollutant, aggregation level, and year - no login needed
+- For a filtered slice, use [Download Daily Data](https://www.epa.gov/outdoor-air-quality-data/download-daily-data); for programmatic access, register for the [AQS API](https://aqs.epa.gov/aqsweb/documents/data_api.html)
+#### Database Time Range
+- 1980-2026
+	- Scattered AQS records reach back to 1957 for a few Los Angeles County monitors; 1980 marks the start of nationally consistent monitoring procedures
+#### Access Type
+- Public
+#### Citation Information
+- Follow the instructions on [How do I cite AirData?](https://www.epa.gov/outdoor-air-quality-data/how-do-i-cite-data-and-graphics-obtained-airdata-website)
+- US Environmental Protection Agency. *Air Quality System Data Mart* [internet database], available via &lt;https://www.epa.gov/outdoor-air-quality-data&gt;. Accessed September 1, 2026.
+- See specific source citation details on the database website.</t>
+        </is>
+      </c>
+      <c r="N44" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="O44" s="1" t="n"/>
       <c r="P44" s="1" t="n"/>
       <c r="Q44" s="1" t="n"/>
@@ -4378,20 +4509,84 @@
       <c r="AB44" s="2" t="n"/>
     </row>
     <row r="45" ht="14.25" customHeight="1">
-      <c r="A45" s="1" t="n"/>
-      <c r="B45" s="1" t="n"/>
-      <c r="C45" s="1" t="n"/>
-      <c r="D45" s="3" t="n"/>
-      <c r="E45" s="1" t="n"/>
-      <c r="F45" s="1" t="n"/>
-      <c r="G45" s="1" t="n"/>
+      <c r="A45" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>Water Quality Portal</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>Water Quality Portal serves 400+ million water-quality records from USGS, EPA, and 1,000+ partners for research.</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.waterqualitydata.us/</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>Ecosystems; Animals; People</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>United States; Global</t>
+        </is>
+      </c>
       <c r="H45" s="1" t="n"/>
-      <c r="I45" s="1" t="n"/>
-      <c r="J45" s="1" t="n"/>
-      <c r="K45" s="3" t="n"/>
-      <c r="L45" s="1" t="n"/>
-      <c r="M45" s="3" t="n"/>
-      <c r="N45" s="1" t="n"/>
+      <c r="I45" s="1" t="n">
+        <v>1900</v>
+      </c>
+      <c r="J45" s="1" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Water Quality; Ecosystem Data; Public Health; Conservation; Agriculture; Wildlife</t>
+        </is>
+      </c>
+      <c r="L45" s="1" t="inlineStr">
+        <is>
+          <t>Water Quality Portal; WQP; waterqualitydata.us; USGS; U.S. Geological Survey; United States Geological Survey; EPA; U.S. Environmental Protection Agency; Environmental Protection Agency; NWQMC; National Water Quality Monitoring Council; USDA; Agricultural Research Service; ARS; STEWARDS; NWIS; National Water Information System; WQX; Water Quality Exchange; WQX 3.0; STORET; BIODATA; BioData; water quality; water data; freshwater; surface water; groundwater; drinking water; source water; streams; rivers; lakes; reservoirs; estuaries; coastal waters; wetlands; wells; springs; aquifers; watershed; nutrients; nitrogen; phosphorus; nitrate; phosphate; pH; dissolved oxygen; water temperature; specific conductance; conductivity; turbidity; salinity; metals; heavy metals; mercury; pesticides; contaminants; pollutants; sediment; chlorophyll; E. coli; fecal coliform; fecal indicator bacteria; pathogens; microbiology; biological indicators; macroinvertebrates; benthic; fish community; habitat assessment; taxonomy; aquatic life; aquatic ecology; limnology; hydrology; watershed science; water resources; water monitoring; water sampling; discrete sampling; monitoring stations; monitoring network; water-quality assessment; biogeochemistry; CSV; TSV; Excel; XLSX; KML; KMZ; GeoJSON; XML; WQX XML; REST API; web services; WMS; WFS; OGC; dataRetrieval; R package; R; Python; United States; all 50 states; District of Columbia; Puerto Rico; Guam; American Samoa; Canada; Mexico; Great Lakes; HUC; hydrologic unit code; bounding box; county-level; state-level; Water Quality; Ecosystem Data; Public Health; Conservation; Agriculture; Wildlife; Historic; Current; Present; 1900-2026; twice-weekly updates; century-scale records</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>The Water Quality Portal (WQP) is the largest standardized source of discrete water-quality monitoring data for the United States, integrating the USGS National Water Information System (NWIS), the EPA Water Quality Exchange (WQX), the USDA ARS STEWARDS database, and USGS BioData into a single query point. It delivers physical, chemical, microbiological, and biological results - nutrients, contaminants, pH, temperature, bacteria, and aquatic-community metrics - from millions of monitoring locations in streams, lakes, groundwater, and coastal waters, with some records extending back more than a century. USGS NWIS data is refreshed daily and EPA WQX data weekly (Thursday evenings), and the portal is midway through a multi-year modernization to the richer WQX 3.0 data profile.
+#### Host Organization
+- United States Geological Survey (USGS), U.S. Environmental Protection Agency (EPA), and the National Water Quality Monitoring Council (NWQMC)
+#### Data Format
+- Query downloads: **CSV**, **TSV**, **MS Excel**, **KML/KMZ**, **GeoJSON**, and **WQX XML**, optionally zipped
+- REST-like web services (Station, Result, Project, Activity, and biological endpoints) plus OGC WMS/WFS map services; the USGS *dataRetrieval* R package wraps them
+#### How to access data of interest
+- Open the [Water Quality Portal](https://www.waterqualitydata.us/) and build a query by location, site type, sample media, characteristic, and date range
+- Choose a data profile and file format, then download; guidance in the [WQP User Guide](https://www.waterqualitydata.us/portal_userguide/)
+- For scripted retrieval, see the [Web Services Guide](https://www.waterqualitydata.us/webservices_documentation/); USGS data added after March 11, 2024 currently requires the [WQX 3.0 beta profiles](https://www.waterqualitydata.us/beta/)
+#### Database Time Range
+- 1900-2026
+	- Holdings date back more than a century; no exact earliest year is published
+#### Access Type
+- Public
+#### Citation Information
+- Follow the instructions in the [WQP User Guide](https://www.waterqualitydata.us/portal_userguide/) under "Cite the Water Quality Portal"
+- National Water Quality Monitoring Council, United States Geological Survey (USGS), and Environmental Protection Agency (EPA). "Water Quality Portal." *Water Quality Portal*, 2021, &lt;https://doi.org/10.5066/P9QRKUVJ&gt;. 2026-09-01
+- See specific source citation details on the database website.</t>
+        </is>
+      </c>
+      <c r="N45" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="O45" s="1" t="n"/>
       <c r="P45" s="1" t="n"/>
       <c r="Q45" s="1" t="n"/>

</xml_diff>